<commit_message>
feat: geolocation connexions + approbation inscriptions + admin dans header
</commit_message>
<xml_diff>
--- a/exports/risques_meteo.xlsx
+++ b/exports/risques_meteo.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,7 +462,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-03-23 15:04:25</t>
+          <t>2026-04-09 09:47:42</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -472,28 +472,68 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Wed 25/03</t>
+          <t>Sat 11/04</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.4°C</t>
+          <t>7.0°C</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>10.8°C</t>
+          <t>15.8°C</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>8.4 mm</t>
+          <t>10.33 mm</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>3.7</v>
+        <v>3.75</v>
       </c>
       <c r="H2" t="inlineStr">
+        <is>
+          <t>🌧️ Alerte pluie</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-04-09 09:47:42</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Clairoix 🏣</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sat 11/04</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>6.8°C</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>17.0°C</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>9.05 mm</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>🌧️ Alerte pluie</t>
         </is>

</xml_diff>